<commit_message>
Sync current Scout guide, firmware, Faces and v8 cases
</commit_message>
<xml_diff>
--- a/01-Electronics-CarrierC/C3-Carrier-RevC-BOM.xlsx
+++ b/01-Electronics-CarrierC/C3-Carrier-RevC-BOM.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Carrier C BOM" sheetId="1" r:id="Rd037db921db04d2c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Carrier C BOM" sheetId="1" r:id="R9aad5983f75d4250"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -343,7 +343,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="2" t="str">
-        <x:v>46 fitted components / 56 ECAD references / reviewed 2026-10-04</x:v>
+        <x:v>46 fitted components / 45 factory assembly / 1 user module / reviewed 2026-10-05</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -555,26 +555,26 @@
         <x:v>SOT-23-6</x:v>
       </x:c>
       <x:c r="E11" s="12" t="str">
-        <x:v>Fortune</x:v>
+        <x:v>PUOLOP</x:v>
       </x:c>
       <x:c r="F11" s="12" t="str">
-        <x:v>DW01A-G</x:v>
+        <x:v>DW01A</x:v>
       </x:c>
       <x:c r="G11" s="12" t="str">
-        <x:v>C61503</x:v>
+        <x:v>C351410</x:v>
       </x:c>
       <x:c r="H11" s="12" t="str">
         <x:v>Extended</x:v>
       </x:c>
       <x:c r="I11" s="12" t="str">
-        <x:v>JLC catalog confirmed; LCSC reports unavailable</x:v>
+        <x:v>JLC stock verified 2026-10-05; user selected</x:v>
       </x:c>
       <x:c r="J11" s="2"/>
       <x:c r="K11" s="10" t="str">
-        <x:v>https://jlcpcb.com/partdetail/FortuneSemicon-DW01AG/C61503</x:v>
+        <x:v>https://jlcpcb.com/partdetail/DW01A/C351410</x:v>
       </x:c>
       <x:c r="L11" s="10" t="str">
-        <x:v>Source or pre-order exact part. Do not substitute DW01+ without reviewing thresholds.</x:v>
+        <x:v>Pin-compatible SOT-23-6; 2.5 V cutoff / 2.9 V recovery, 150 mV current sense. Allows 0 V battery charging; verify protection behavior.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="36" customHeight="1">
@@ -591,26 +591,26 @@
         <x:v>TSSOP-8</x:v>
       </x:c>
       <x:c r="E12" s="4" t="str">
-        <x:v>Fortune</x:v>
+        <x:v>TECH PUBLIC</x:v>
       </x:c>
       <x:c r="F12" s="4" t="str">
-        <x:v>FS8205A</x:v>
+        <x:v>8205A</x:v>
       </x:c>
       <x:c r="G12" s="4" t="str">
-        <x:v>C14212</x:v>
+        <x:v>C7419210</x:v>
       </x:c>
       <x:c r="H12" s="4" t="str">
         <x:v>Extended</x:v>
       </x:c>
       <x:c r="I12" s="4" t="str">
-        <x:v>JLC catalog confirmed; stock not verified</x:v>
+        <x:v>JLC stock verified 2026-10-05; user selected</x:v>
       </x:c>
       <x:c r="J12" s="2"/>
       <x:c r="K12" s="10" t="str">
-        <x:v>https://jlcpcb.com/partdetail/LCSC-FS8205A/C14212</x:v>
+        <x:v>https://jlcpcb.com/partdetail/TECHPUBLIC-8205A/C7419210</x:v>
       </x:c>
       <x:c r="L12" s="10" t="str">
-        <x:v>Exact Fortune TSSOP-8 pinout. SOT-23-6 parts sharing the name are not equivalent.</x:v>
+        <x:v>TSSOP-8, common drain at pins 1/8. Lower RDS(on) raises overcurrent trip current; verify prototype protection.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="36" customHeight="1">
@@ -882,21 +882,23 @@
         <x:v>Panasonic</x:v>
       </x:c>
       <x:c r="F20" s="4" t="str">
-        <x:v>EEUFR1E101</x:v>
-      </x:c>
-      <x:c r="G20" s="4" t="str"/>
+        <x:v>EEUFM1E101</x:v>
+      </x:c>
+      <x:c r="G20" s="4" t="str">
+        <x:v>C713389</x:v>
+      </x:c>
       <x:c r="H20" s="4" t="str">
-        <x:v>Hand solder</x:v>
+        <x:v>THT assembly</x:v>
       </x:c>
       <x:c r="I20" s="4" t="str">
-        <x:v>Manufacturer dimensions verified; distributor quote required</x:v>
+        <x:v>JLC: 1130 in stock; 1097 orderable on 2026-10-05</x:v>
       </x:c>
       <x:c r="J20" s="2"/>
       <x:c r="K20" s="10" t="str">
-        <x:v>https://industrial.panasonic.com/kr/products/pt/aluminum-cap-lead/models/EEUFR1E101</x:v>
+        <x:v>https://jlcpcb.com/partdetail/PANASONIC-EEUFM1E101/C713389</x:v>
       </x:c>
       <x:c r="L20" s="10" t="str">
-        <x:v>Positive pad 1. 455 mA rms ripple at 100 kHz; 130 mohm impedance max.</x:v>
+        <x:v>FM substitutes FR: same 100 uF/25 V, 6.3 x 11.2 mm, 2.5 mm pitch, 455 mA ripple and 130 mohm impedance. Endurance 2000 h vs 5000 h at 105 C. Pad 1 positive. JLC wave soldering; Economic/Standard supported.</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="36" customHeight="1">
@@ -1283,30 +1285,32 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C32" s="4" t="str">
-        <x:v>USB-C power input</x:v>
+        <x:v>USB-C charging inlet</x:v>
       </x:c>
       <x:c r="D32" s="4" t="str">
-        <x:v>USB4125 custom round-stake footprint</x:v>
+        <x:v>USB-C-SHOUHAN-6P-C456012</x:v>
       </x:c>
       <x:c r="E32" s="4" t="str">
-        <x:v>GCT</x:v>
+        <x:v>SHOU HAN</x:v>
       </x:c>
       <x:c r="F32" s="4" t="str">
-        <x:v>USB4125-GF-A-0190</x:v>
-      </x:c>
-      <x:c r="G32" s="4" t="str"/>
+        <x:v>TYPE-C 6P</x:v>
+      </x:c>
+      <x:c r="G32" s="4" t="str">
+        <x:v>C456012</x:v>
+      </x:c>
       <x:c r="H32" s="4" t="str">
-        <x:v>Hand solder</x:v>
+        <x:v>Extended</x:v>
       </x:c>
       <x:c r="I32" s="4" t="str">
-        <x:v>Manufacturer part selected; JLC listing not found</x:v>
+        <x:v>JLC stock verified 2026-10-05; user selected</x:v>
       </x:c>
       <x:c r="J32" s="2"/>
       <x:c r="K32" s="10" t="str">
-        <x:v>https://gct.co/connector/usb4125</x:v>
+        <x:v>https://jlcpcb.com/partdetail/C456012</x:v>
       </x:c>
       <x:c r="L32" s="10" t="str">
-        <x:v>Round 1.35 mm shell holes retained. Trial-fit connector before ordering boards; manufacturer drawing specifies slots.</x:v>
+        <x:v>6-contact power-only 5 V / 3 A. Footprint updated in Fusion board v9: four 0.60 x 1.40 mm plated slots, 1.00 x 1.80 mm copper lands; body-center placement 28.6,24 mm, R90. Factory SMT assembly; 3000 mating cycles.</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="36" customHeight="1">
@@ -1374,7 +1378,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcf127d15c2dc4277"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd9a856b31e424c60"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>